<commit_message>
Correction suite à la revue c7e476aa2e435ab16c60bd61301a006b63ac23ae
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-bundle-document.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-bundle-document.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-04T16:07:16+00:00</t>
+    <t>2025-03-06T10:23:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>FrBundleDocument permet d’assembler les éléments de l’en-tête et du corps d’un document.</t>
+    <t>Ce profil permet d’assembler les éléments de l’en-tête et du corps d’un document.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
Corrections après revues 381d1cffd6d68f69ebfa409e1bb84ab612ca8a11
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-bundle-document.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-bundle-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-31T09:17:15+00:00</t>
+    <t>2025-04-14T15:21:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -262,10 +262,10 @@
 </t>
   </si>
   <si>
-    <t>Bundle Document</t>
-  </si>
-  <si>
-    <t>Bundle Document.</t>
+    <t>Contains a collection of resources</t>
+  </si>
+  <si>
+    <t>A container for a collection of resources.</t>
   </si>
   <si>
     <t>bdl-1:total only when a search or history {total.empty() or (type = 'searchset') or (type = 'history')}
@@ -573,7 +573,7 @@
     <t>Bundle.entry</t>
   </si>
   <si>
-    <t>8</t>
+    <t>7</t>
   </si>
   <si>
     <t>Ressource Entry dans le FrBundleDocument</t>
@@ -892,10 +892,10 @@
 </t>
   </si>
   <si>
-    <t>Clinical document</t>
-  </si>
-  <si>
-    <t>Clinical document.</t>
+    <t>A set of resources composed into a single coherent clinical statement with clinical attestation</t>
+  </si>
+  <si>
+    <t>A set of healthcare-related information that is assembled together into a single logical package that provides a single coherent statement of meaning, establishes its own context and that has clinical attestation with regard to who is making the statement. A Composition defines the structure and narrative content necessary for a document. However, a Composition alone does not constitute a document. Rather, the Composition must be the first entry in a Bundle where Bundle.type=document, and any other resources referenced from Composition must be included as subsequent entries in the Bundle (for example Patient, Practitioner, Encounter, etc.).</t>
   </si>
   <si>
     <t>While the focus of this specification is on patient-specific clinical statements, this resource can also apply to other healthcare-related statements such as study protocol designs, healthcare invoices and other activities that are not necessarily patient-specific or clinical.</t>
@@ -36724,7 +36724,7 @@
       </c>
       <c r="E305" s="2"/>
       <c r="F305" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G305" t="s" s="2">
         <v>79</v>

</xml_diff>